<commit_message>
Draft_107: full-pass indicate audit; Aas3 indicates EC; totals 65/65
</commit_message>
<xml_diff>
--- a/thesis/007_CompiledResult_Draft_020.xlsx
+++ b/thesis/007_CompiledResult_Draft_020.xlsx
@@ -958,7 +958,7 @@
         </is>
       </c>
       <c r="G18" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="19">
@@ -1683,7 +1683,7 @@
         </is>
       </c>
       <c r="G43" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="44">
@@ -1991,10 +1991,10 @@
         <v>296</v>
       </c>
       <c r="D54" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E54" t="n">
-        <v>0.68</v>
+        <v>1.01</v>
       </c>
       <c r="F54" t="inlineStr">
         <is>
@@ -2219,7 +2219,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I65"/>
+  <dimension ref="A1:I66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4680,7 +4680,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Aas4</t>
+          <t>Aas3</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -4688,17 +4688,14 @@
           <t>Agriculture</t>
         </is>
       </c>
-      <c r="C58" t="n">
-        <v>7</v>
-      </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>The statistical analysis suggests that there is no significant difference among the treatments with regard to their initial weight, gain in weight, average daily gain, and feed conversion ratio of the experimental rabbits.</t>
+          <t>This indicates that ducks fed with 100% commercial feeds rice bran mixed with golden apple snail performed better in final weight, gain, and feed conversion ratio.</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>suggests</t>
+          <t>indicates</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
@@ -4712,18 +4709,18 @@
         </is>
       </c>
       <c r="H58" t="n">
-        <v>161</v>
+        <v>296</v>
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>Lexical hedge: 'The statistical analysis suggests that there is no significant difference among the treatments' = introduces finding.</t>
+          <t>[FULL-PASS ADD] Lexical hedge: 'This indicates that... performed better' — inference from significant differences to comparative performance claim, not operational restatement of a metric definition. Working Test: removal raises commitment to the performance claim.</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Aas5</t>
+          <t>Aas4</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -4732,21 +4729,21 @@
         </is>
       </c>
       <c r="C59" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Fortunately, insect farming can be seen as a potential solution for filling the protein gap for feed and food resources in a more sustainable manned compared to other animal protein sources.</t>
+          <t>The statistical analysis suggests that there is no significant difference among the treatments with regard to their initial weight, gain in weight, average daily gain, and feed conversion ratio of the experimental rabbits.</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>can</t>
+          <t>suggests</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>Modal Verbs</t>
+          <t>Lexical Hedges</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
@@ -4755,11 +4752,11 @@
         </is>
       </c>
       <c r="H59" t="n">
-        <v>316</v>
+        <v>161</v>
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>Modal hedge: 'insect farming can be seen as a potential solution'.</t>
+          <t>Lexical hedge: 'The statistical analysis suggests that there is no significant difference among the treatments' = introduces finding.</t>
         </is>
       </c>
     </row>
@@ -4784,12 +4781,12 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>potential</t>
+          <t>can</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>Lexical Hedges</t>
+          <t>Modal Verbs</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
@@ -4802,14 +4799,14 @@
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>[AMB] Lexical hedge (Working Test): removing 'potential' changes commitment  -  'a solution' is stronger endorsement than 'a potential solution'. Multi-hedge isolation: 'can' already coded EC in same sentence; 'potential' independently softens.</t>
+          <t>Modal hedge: 'insect farming can be seen as a potential solution'.</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Aas7</t>
+          <t>Aas5</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -4818,16 +4815,16 @@
         </is>
       </c>
       <c r="C61" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Statistical analysis showed that there was no significant difference but showed numerical trends among the treatments in relation to initial weight, final weight, gain in weight, average daily gain, dry matter intake, and feed conversion ratio of the experimental rabbits In conclusion, all treatments are comparable in terms of growth, implying that Fermented Madre de Agua is a viable feed component under these conditions.</t>
+          <t>Fortunately, insect farming can be seen as a potential solution for filling the protein gap for feed and food resources in a more sustainable manned compared to other animal protein sources.</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>implying</t>
+          <t>potential</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
@@ -4841,11 +4838,11 @@
         </is>
       </c>
       <c r="H61" t="n">
-        <v>202</v>
+        <v>316</v>
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>Lexical hedge: 'implying that Fermented Madre de Agua is a viable feed component' = inferential conclusion.</t>
+          <t>[AMB] Lexical hedge (Working Test): removing 'potential' changes commitment  -  'a solution' is stronger endorsement than 'a potential solution'. Multi-hedge isolation: 'can' already coded EC in same sentence; 'potential' independently softens.</t>
         </is>
       </c>
     </row>
@@ -4861,21 +4858,21 @@
         </is>
       </c>
       <c r="C62" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Feeding 20% fermented Madre De Agua may improve final weight, while feeding 10% fermented Madre De Agua may reduce dry matter intake.</t>
+          <t>Statistical analysis showed that there was no significant difference but showed numerical trends among the treatments in relation to initial weight, final weight, gain in weight, average daily gain, dry matter intake, and feed conversion ratio of the experimental rabbits In conclusion, all treatments are comparable in terms of growth, implying that Fermented Madre de Agua is a viable feed component under these conditions.</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>may</t>
+          <t>implying</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>Modal Verbs</t>
+          <t>Lexical Hedges</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
@@ -4888,7 +4885,7 @@
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>Modal hedge: 'Feeding 20% fermented Madre De Agua may improve final weight' possibility claim.</t>
+          <t>Lexical hedge: 'implying that Fermented Madre de Agua is a viable feed component' = inferential conclusion.</t>
         </is>
       </c>
     </row>
@@ -4931,14 +4928,14 @@
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>Modal hedge: 'feeding 10% fermented Madre De Agua may reduce dry matter intake' possibility claim.</t>
+          <t>Modal hedge: 'Feeding 20% fermented Madre De Agua may improve final weight' possibility claim.</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Aas10</t>
+          <t>Aas7</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -4947,16 +4944,16 @@
         </is>
       </c>
       <c r="C64" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>In conclusion, based on the results, it can be stated that the ratio of 70% guinea grass (GG) + 30% concentrate (C), the control group, had a significantly higher (P&lt;0.01) feed conversion ratio, while rabbits in treatment T3 (50% guinea grass, 20% azolla, and 30% concentrate) had a significantly higher (P&lt;0.01) dry matter intake.</t>
+          <t>Feeding 20% fermented Madre De Agua may improve final weight, while feeding 10% fermented Madre De Agua may reduce dry matter intake.</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>can</t>
+          <t>may</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
@@ -4970,11 +4967,11 @@
         </is>
       </c>
       <c r="H64" t="n">
-        <v>283</v>
+        <v>202</v>
       </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t>Modal hedge: 'it can be stated that the ratio of 70% guinea grass (GG) + 30% concentrate (C)... had a significantly higher feed conversion ratio'. Same sentence as DO frame 'In conclusion' (P/DO log). Frame is DO; can is the modal under review for claim weight. Not a co-label.</t>
+          <t>Modal hedge: 'feeding 10% fermented Madre De Agua may reduce dry matter intake' possibility claim.</t>
         </is>
       </c>
     </row>
@@ -4990,21 +4987,21 @@
         </is>
       </c>
       <c r="C65" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>The researchers also saw that the treatment of 50% Guinea grass + 20% Azolla + 30% concentrates has potential as an alternative feed ration for rabbits without adverse effects, and considering that azolla can help breeders to lessen the feed cost in production.</t>
+          <t>In conclusion, based on the results, it can be stated that the ratio of 70% guinea grass (GG) + 30% concentrate (C), the control group, had a significantly higher (P&lt;0.01) feed conversion ratio, while rabbits in treatment T3 (50% guinea grass, 20% azolla, and 30% concentrate) had a significantly higher (P&lt;0.01) dry matter intake.</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>potential</t>
+          <t>can</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>Lexical Hedges</t>
+          <t>Modal Verbs</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
@@ -5016,6 +5013,49 @@
         <v>283</v>
       </c>
       <c r="I65" t="inlineStr">
+        <is>
+          <t>Modal hedge: 'it can be stated that the ratio of 70% guinea grass (GG) + 30% concentrate (C)... had a significantly higher feed conversion ratio'. Same sentence as DO frame 'In conclusion' (P/DO log). Frame is DO; can is the modal under review for claim weight. Not a co-label.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Aas10</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Agriculture</t>
+        </is>
+      </c>
+      <c r="C66" t="n">
+        <v>10</v>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>The researchers also saw that the treatment of 50% Guinea grass + 20% Azolla + 30% concentrates has potential as an alternative feed ration for rabbits without adverse effects, and considering that azolla can help breeders to lessen the feed cost in production.</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>potential</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>Lexical Hedges</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>EC</t>
+        </is>
+      </c>
+      <c r="H66" t="n">
+        <v>283</v>
+      </c>
+      <c r="I66" t="inlineStr">
         <is>
           <t>Lexical hedge (claim in conclusion): 'has potential as an alternative feed ration for rabbits' qualifies the claim about implications.</t>
         </is>
@@ -5032,7 +5072,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I64"/>
+  <dimension ref="A1:I66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7466,6 +7506,70 @@
       <c r="I64" t="inlineStr">
         <is>
           <t>FP-Cap. Can + promote: capability. Suggest coded separately as Lexical EC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Acs2</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Agriculture</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>The result of the study indicate that there were no statistically significant differences observed across the various measured parameters for the two treatments.</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>indicate</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>FP-Gen</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>[FULL-PASS ADD] Factive reporting of NS statistical result — parallel to other 'results indicate that [stat finding]' FP-Gen cases.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>B17</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Biology</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>The findings indicate that P. propinquum fruit ethanolic extract contains bioactive compounds with antioxidant and selective antibacterial properties.</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>indicate</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>FP-Gen</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>[FULL-PASS ADD] Factive reporting of composition/activity findings — evidential pointer restating what assays showed, not a hedged inference beyond the data.</t>
         </is>
       </c>
     </row>
@@ -7522,7 +7626,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="5">
@@ -7532,7 +7636,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>63</v>
+        <v>65</v>
       </c>
     </row>
     <row r="6">
@@ -7542,7 +7646,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.46</v>
+        <v>0.47</v>
       </c>
     </row>
     <row r="7">
@@ -7592,7 +7696,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>37</v>
+        <v>39</v>
       </c>
     </row>
     <row r="12">
@@ -7612,7 +7716,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="14">
@@ -7632,7 +7736,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="16">
@@ -7666,7 +7770,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Draft_020 full-pass inventory. Retained EC = curated 64 (Draft_107 after Acs9 can→FP-Cap).</t>
+          <t>Draft_020 full-pass: +Aas3 indicates EC; +Acs2/B17 indicate FP-Gen. Retained 65, FP 65. Indicating: EC when inference beyond data; FP-Gen when evidential restatement.</t>
         </is>
       </c>
     </row>

</xml_diff>